<commit_message>
complete package punm y add img
</commit_message>
<xml_diff>
--- a/Docs/Resources/Documents/ProjectBudget.xlsx
+++ b/Docs/Resources/Documents/ProjectBudget.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julit\source\Projects\ClimbEdge\Docs\Estimate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julio.castro904\Documents\codigos\personal\ClimbEdge\Docs\Resources\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7CE817B-6983-4EE3-9A2A-22E798143D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5AE2592-CEB7-4133-9100-D710BF487CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5443361D-16A8-4F27-B5AC-62FADFB7C971}"/>
+    <workbookView xWindow="6000" yWindow="4890" windowWidth="18885" windowHeight="8820" xr2:uid="{5443361D-16A8-4F27-B5AC-62FADFB7C971}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>Nombre</t>
   </si>
@@ -121,6 +121,12 @@
   </si>
   <si>
     <t>Colchoneta</t>
+  </si>
+  <si>
+    <t>soldadura</t>
+  </si>
+  <si>
+    <t>Soldada de pines del rpi</t>
   </si>
 </sst>
 </file>
@@ -128,7 +134,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -165,29 +171,30 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
     <dxf>
-      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -215,7 +222,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="34" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+      <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     </dxf>
     <dxf>
       <font>
@@ -264,8 +271,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EF5ABBDF-1FEA-429C-AE86-38CF263D3E2A}" name="Table1" displayName="Table1" ref="A1:G13" totalsRowCount="1" headerRowDxfId="10">
-  <autoFilter ref="A1:G12" xr:uid="{EF5ABBDF-1FEA-429C-AE86-38CF263D3E2A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{EF5ABBDF-1FEA-429C-AE86-38CF263D3E2A}" name="Table1" displayName="Table1" ref="A1:G14" totalsRowCount="1" headerRowDxfId="10">
+  <autoFilter ref="A1:G13" xr:uid="{EF5ABBDF-1FEA-429C-AE86-38CF263D3E2A}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{5AAFB984-C85B-4BF1-A918-1C571672DC61}" name="#" totalsRowLabel="Total">
       <calculatedColumnFormula>ROW()-2</calculatedColumnFormula>
@@ -274,8 +281,8 @@
     <tableColumn id="3" xr3:uid="{C86D0AB4-DEB6-40A8-9392-93A7487C0EE6}" name="Descripción" dataDxfId="8" totalsRowDxfId="2"/>
     <tableColumn id="9" xr3:uid="{F216D570-7ECE-4417-99A9-CCD3AF39DFEE}" name="Link" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{30834DA3-1966-47EB-8A17-1138734385AE}" name="Cantidad" dataDxfId="6" totalsRowDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{E683EF20-9F04-489F-B245-87EE163DBC3E}" name="Valor" dataDxfId="5" dataCellStyle="Currency"/>
-    <tableColumn id="6" xr3:uid="{6CBFF6F8-BBF0-4390-82B5-2CCADAAB1B96}" name="Valor Total" totalsRowFunction="custom" dataDxfId="4" totalsRowDxfId="0" dataCellStyle="Currency">
+    <tableColumn id="5" xr3:uid="{E683EF20-9F04-489F-B245-87EE163DBC3E}" name="Valor" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{6CBFF6F8-BBF0-4390-82B5-2CCADAAB1B96}" name="Valor Total" totalsRowFunction="custom" dataDxfId="4" totalsRowDxfId="0">
       <calculatedColumnFormula>Table1[[#This Row],[Cantidad]]*Table1[[#This Row],[Valor]]</calculatedColumnFormula>
       <totalsRowFormula>SUM(Table1[Valor Total])</totalsRowFormula>
     </tableColumn>
@@ -285,7 +292,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -601,19 +608,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CFC82DF-8B66-42C3-911C-E89DA602034C}">
-  <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.77734375" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" style="4" customWidth="1"/>
-    <col min="3" max="3" width="35.5546875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="5.109375" customWidth="1"/>
-    <col min="5" max="5" width="8.77734375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.33203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="35.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="5.140625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.28515625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="4" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>7</v>
       </c>
@@ -636,7 +643,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A2">
         <f t="shared" ref="A2:A8" si="0">ROW()-2</f>
         <v>0</v>
@@ -655,7 +662,7 @@
         <v>22.31</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>1</v>
@@ -677,7 +684,7 @@
         <v>22.07</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -699,7 +706,7 @@
         <v>9.9499999999999993</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -721,7 +728,7 @@
         <v>21.99</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -743,7 +750,7 @@
         <v>11.99</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -765,7 +772,7 @@
         <v>9.99</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -787,7 +794,7 @@
         <v>20.99</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <f t="shared" ref="A9:A10" si="1">ROW()-2</f>
         <v>7</v>
@@ -809,7 +816,7 @@
         <v>50.099999999999994</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <f t="shared" si="1"/>
         <v>8</v>
@@ -831,7 +838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <f>ROW()-2</f>
         <v>9</v>
@@ -845,7 +852,7 @@
       <c r="E11" s="2">
         <v>0</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11" s="8">
         <v>1.25</v>
       </c>
       <c r="G11" s="1">
@@ -853,7 +860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <f>ROW()-2</f>
         <v>10</v>
@@ -861,23 +868,45 @@
       <c r="B12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="6"/>
       <c r="E12" s="2">
         <v>1</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="1">
         <f>Table1[[#This Row],[Cantidad]]*Table1[[#This Row],[Valor]]</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <f>ROW()-2</f>
+        <v>11</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="1">
+        <v>5</v>
+      </c>
+      <c r="G13" s="7">
+        <f>Table1[[#This Row],[Cantidad]]*Table1[[#This Row],[Valor]]</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>6</v>
       </c>
-      <c r="F13"/>
-      <c r="G13" s="3">
+      <c r="F14"/>
+      <c r="G14" s="3">
         <f>SUM(Table1[Valor Total])</f>
-        <v>169.39</v>
+        <v>174.39</v>
       </c>
     </row>
   </sheetData>
@@ -895,7 +924,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F716EC4A-8D85-4EC7-9E68-DC17C6701E4E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add ing en some docs
</commit_message>
<xml_diff>
--- a/Docs/Resources/Documents/ProjectBudget.xlsx
+++ b/Docs/Resources/Documents/ProjectBudget.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julio.castro904\Documents\codigos\personal\ClimbEdge\Docs\Resources\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5AE2592-CEB7-4133-9100-D710BF487CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D70D1F-DDE2-4D3F-B0CD-D591B663D672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="4890" windowWidth="18885" windowHeight="8820" xr2:uid="{5443361D-16A8-4F27-B5AC-62FADFB7C971}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5443361D-16A8-4F27-B5AC-62FADFB7C971}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -173,7 +173,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -184,8 +184,6 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -828,14 +826,14 @@
         <v>11</v>
       </c>
       <c r="E10" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F10" s="1">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G10" s="1">
         <f>Table1[[#This Row],[Cantidad]]*Table1[[#This Row],[Valor]]</f>
-        <v>0</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -852,7 +850,7 @@
       <c r="E11" s="2">
         <v>0</v>
       </c>
-      <c r="F11" s="8">
+      <c r="F11" s="6">
         <v>1.25</v>
       </c>
       <c r="G11" s="1">
@@ -887,14 +885,13 @@
       <c r="C13" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="6"/>
       <c r="E13" s="2">
         <v>1</v>
       </c>
       <c r="F13" s="1">
         <v>5</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="1">
         <f>Table1[[#This Row],[Cantidad]]*Table1[[#This Row],[Valor]]</f>
         <v>5</v>
       </c>
@@ -906,7 +903,7 @@
       <c r="F14"/>
       <c r="G14" s="3">
         <f>SUM(Table1[Valor Total])</f>
-        <v>174.39</v>
+        <v>294.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>